<commit_message>
feat: implement RAG pipeline with vector storage, document loaders, and multi-agent system for task orchestration and assessment
</commit_message>
<xml_diff>
--- a/data/storage/learner_assignments.xlsx
+++ b/data/storage/learner_assignments.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -878,6 +878,41 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>M-92244A</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>L002</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Assignment 4: Version Control &amp; Software Design</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>C001</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2026-05-19 18:23:07</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: implement assessment orchestration logic, evaluation agent, and assignment tracking system
</commit_message>
<xml_diff>
--- a/data/storage/learner_assignments.xlsx
+++ b/data/storage/learner_assignments.xlsx
@@ -481,11 +481,11 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -621,15 +621,20 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
           <t>2026-05-18 15:48:23</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2026-05-19 18:49:01</t>
         </is>
       </c>
     </row>
@@ -726,11 +731,11 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat: implement agentic assignment and progress tracking nodes within the orchestrator graph
</commit_message>
<xml_diff>
--- a/data/storage/learner_assignments.xlsx
+++ b/data/storage/learner_assignments.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -481,15 +481,20 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
           <t>2026-05-18 15:36:44</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2026-05-21 11:33:49</t>
         </is>
       </c>
     </row>
@@ -910,6 +915,41 @@
       <c r="G14" t="inlineStr">
         <is>
           <t>2026-05-19 18:23:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>M-A55A4F</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>L001</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Assignment 8: Data Science &amp; Pandas</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>C001</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>2026-05-20 17:16:32</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: implement orchestrator nodes and agent framework for AI-driven learner assistance
</commit_message>
<xml_diff>
--- a/data/storage/learner_assignments.xlsx
+++ b/data/storage/learner_assignments.xlsx
@@ -481,15 +481,20 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
           <t>2026-05-18 15:36:44</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2026-05-19 19:09:46</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: implement MCP server for learner management and initialize agentic orchestrator nodes and configuration
</commit_message>
<xml_diff>
--- a/data/storage/learner_assignments.xlsx
+++ b/data/storage/learner_assignments.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -485,7 +485,7 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -494,7 +494,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-05-19 19:09:46</t>
+          <t>2026-05-21 17:54:35</t>
         </is>
       </c>
     </row>
@@ -591,15 +591,20 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
           <t>2026-05-18 15:42:07</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2026-05-21 16:41:09</t>
         </is>
       </c>
     </row>
@@ -731,7 +736,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="F9" t="n">
@@ -740,6 +745,11 @@
       <c r="G9" t="inlineStr">
         <is>
           <t>2026-05-18 15:50:50</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>2026-05-21 17:45:12</t>
         </is>
       </c>
     </row>
@@ -915,6 +925,636 @@
       <c r="G14" t="inlineStr">
         <is>
           <t>2026-05-19 18:23:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>M-0FCC7D</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>L002</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Assignment 7: Docker &amp; Infrastructure</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>C001</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>2026-05-21 18:35:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>M-36B5E4</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>L001</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Assignment 3: Systems &amp; Networking</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>C001</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>2026-05-21 18:48:49</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>M-113E5E</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>L001</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Assignment 5: Relational Databases &amp; SQL</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>C001</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>2026-05-21 18:48:52</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>M-7149C6</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>L001</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Assignment 6: API Development with FastAPI</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>C001</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2026-05-21 18:48:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>M-D6FF23</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>L001</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Assignment 7: Docker &amp; Infrastructure</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>C001</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>2026-05-21 18:48:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>M-EA5A1D</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>L001</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Assignment 8: Data Science &amp; Pandas</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>C001</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>2026-05-21 18:48:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>M-525CDC</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>L001</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Assignment 9: System Design &amp; Architecture</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>C001</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>2026-05-21 18:48:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>M-B06008</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>L001</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Assignment 10: Classical Machine Learning</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>C001</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>2026-05-21 18:49:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>M-8651B7</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>L001</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Assignment 11: Deep Learning &amp; PyTorch</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>C001</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>2026-05-21 18:49:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>M-C573EB</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>L001</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Assignment 12: Prompt Engineering &amp; LLMsn</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>C001</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>2026-05-21 18:49:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>M-0D0361</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>L001</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Assignment 13: Retrieval-Augmented Generation (RAG)</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>C001</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>2026-05-21 18:49:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>M-88B16A</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>L001</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Assignment 15: Model Context Protocol (MCP)</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>C001</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>2026-05-21 18:49:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>M-703E46</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>L002</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Assignment 9: System Design &amp; Architecture</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>C001</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>2026-05-21 18:58:31</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>M-D338FF</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>L003</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Assignment 9: System Design &amp; Architecture</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>C001</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>2026-05-21 18:58:32</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>M-85F48D</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>L002</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Assignment 11: Deep Learning &amp; PyTorch</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>C001</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>2026-05-21 18:59:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>M-38DD9B</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>L003</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Assignment 11: Deep Learning &amp; PyTorch</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>C001</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>2026-05-21 18:59:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>M-5BDD2D</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>L002</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Assignment 5: Relational Databases &amp; SQL</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>C001</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>2026-05-21 18:59:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>M-034F62</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>L003</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Assignment 5: Relational Databases &amp; SQL</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>C001</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>2026-05-21 18:59:11</t>
         </is>
       </c>
     </row>

</xml_diff>